<commit_message>
ingesta: snapshot 2026-07-28 18:44 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-28/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-28/CORDOBA_JUL26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519F75D7-323E-418F-A1EA-7438B1A9E858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8321B3D-F4BF-480D-A547-2690AC87FACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
   <sheets>
     <sheet name="ENERO_2026" sheetId="1" r:id="rId1"/>
@@ -10038,7 +10038,7 @@
                   <c:v>195.6</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-1</c:v>
+                  <c:v>1.7999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>-1</c:v>
@@ -19997,14 +19997,16 @@
       <c r="AD3" s="25">
         <v>40.799999999999997</v>
       </c>
-      <c r="AE3" s="25"/>
+      <c r="AE3" s="25">
+        <v>0.4</v>
+      </c>
       <c r="AF3" s="25"/>
       <c r="AG3" s="25"/>
       <c r="AH3" s="25"/>
       <c r="AI3" s="34"/>
       <c r="AJ3" s="36">
         <f>SUM(E3:AI3)</f>
-        <v>239.40000000000003</v>
+        <v>239.80000000000004</v>
       </c>
       <c r="AK3" s="30">
         <v>27.817857142857147</v>
@@ -20101,7 +20103,9 @@
       <c r="AD4" s="25">
         <v>8.6999999999999993</v>
       </c>
-      <c r="AE4" s="25"/>
+      <c r="AE4" s="25">
+        <v>0</v>
+      </c>
       <c r="AF4" s="25"/>
       <c r="AG4" s="25"/>
       <c r="AH4" s="25"/>
@@ -20205,7 +20209,9 @@
       <c r="AD5" s="25">
         <v>86.5</v>
       </c>
-      <c r="AE5" s="25"/>
+      <c r="AE5" s="25">
+        <v>0</v>
+      </c>
       <c r="AF5" s="25"/>
       <c r="AG5" s="25"/>
       <c r="AH5" s="25"/>
@@ -20309,14 +20315,16 @@
       <c r="AD6" s="25">
         <v>0</v>
       </c>
-      <c r="AE6" s="25"/>
+      <c r="AE6" s="25">
+        <v>1.4</v>
+      </c>
       <c r="AF6" s="25"/>
       <c r="AG6" s="25"/>
       <c r="AH6" s="25"/>
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
         <f t="shared" si="0"/>
-        <v>141.30000000000001</v>
+        <v>142.70000000000002</v>
       </c>
       <c r="AK6" s="30">
         <v>88.719230769230762</v>
@@ -20517,7 +20525,9 @@
       <c r="AD9" s="25">
         <v>0</v>
       </c>
-      <c r="AE9" s="25"/>
+      <c r="AE9" s="25">
+        <v>0</v>
+      </c>
       <c r="AF9" s="25"/>
       <c r="AG9" s="25"/>
       <c r="AH9" s="25"/>
@@ -20697,7 +20707,9 @@
       <c r="AD11" s="25">
         <v>14.2</v>
       </c>
-      <c r="AE11" s="25"/>
+      <c r="AE11" s="25">
+        <v>0</v>
+      </c>
       <c r="AF11" s="25"/>
       <c r="AG11" s="25"/>
       <c r="AH11" s="25"/>
@@ -20799,7 +20811,9 @@
       <c r="AD12" s="25">
         <v>4</v>
       </c>
-      <c r="AE12" s="25"/>
+      <c r="AE12" s="25">
+        <v>0</v>
+      </c>
       <c r="AF12" s="25"/>
       <c r="AG12" s="25"/>
       <c r="AH12" s="25"/>
@@ -20903,7 +20917,9 @@
       <c r="AD13" s="25">
         <v>28</v>
       </c>
-      <c r="AE13" s="25"/>
+      <c r="AE13" s="25">
+        <v>0</v>
+      </c>
       <c r="AF13" s="25"/>
       <c r="AG13" s="25"/>
       <c r="AH13" s="25"/>
@@ -21005,7 +21021,9 @@
       <c r="AD14" s="25">
         <v>0</v>
       </c>
-      <c r="AE14" s="25"/>
+      <c r="AE14" s="25">
+        <v>0</v>
+      </c>
       <c r="AF14" s="25"/>
       <c r="AG14" s="25"/>
       <c r="AH14" s="25"/>
@@ -21109,7 +21127,9 @@
       <c r="AD15" s="25">
         <v>13.4</v>
       </c>
-      <c r="AE15" s="25"/>
+      <c r="AE15" s="25">
+        <v>0</v>
+      </c>
       <c r="AF15" s="25"/>
       <c r="AG15" s="25"/>
       <c r="AH15" s="25"/>
@@ -21330,7 +21350,7 @@
       </c>
       <c r="AE19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>1.7999999999999998</v>
       </c>
       <c r="AF19" s="26">
         <f t="shared" si="1"/>

</xml_diff>